<commit_message>
update metadata file from data folder, final data inventory
</commit_message>
<xml_diff>
--- a/notes/seguimiento_monitoreo.xlsx
+++ b/notes/seguimiento_monitoreo.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Seguimiento" sheetId="1" state="visible" r:id="rId2"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2933" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2931" uniqueCount="656">
   <si>
     <t xml:space="preserve">num_casa</t>
   </si>
@@ -148,7 +148,7 @@
     <t xml:space="preserve">Observaciones octubre 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">DL Tycon octubre 20252</t>
+    <t xml:space="preserve">DL Tycon octubre 2025</t>
   </si>
   <si>
     <t xml:space="preserve">Adrian</t>
@@ -1796,6 +1796,15 @@
     <t xml:space="preserve">11 meses de datos</t>
   </si>
   <si>
+    <t xml:space="preserve">Entrevistas a usuarios   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datos consumo DL nuevos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datos por validar</t>
+  </si>
+  <si>
     <t xml:space="preserve">Actividad</t>
   </si>
   <si>
@@ -1895,25 +1904,19 @@
     <t xml:space="preserve">Se instalaron los 8 dataloggers</t>
   </si>
   <si>
+    <t xml:space="preserve">Trabajo de campo 5 (investigación) - Instalación DL</t>
+  </si>
+  <si>
     <t xml:space="preserve">Se revisaron los DL instalados y se vaciaron datos</t>
   </si>
   <si>
+    <t xml:space="preserve">Trabajo de campo 6 (investigación) - 1er vaciado de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se planea realizar un trabajo de campo de 5 días con los siguientes objetivos: vaciar datos de los dataloggers, recuperar el DL que falta, recabar datos adicionales, realizar un taller/grupo focal, presentación de resultados preliminares. </t>
+  </si>
+  <si>
     <t xml:space="preserve">Visita técnica ENERGETICA - Acondicionamiento de SS - Escuela de Molle Orcko</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trabajo de campo 5 (investigación) - 1er vaciado de datos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enfoque en encuestas CUANTITATIVAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trabajo de campo 5 (investigación) - Seguimiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trabajo de campo 6 (investigación) - Vaciado final de datos y retirado de DL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Posible visita a otras comunidades, para aplicar nuevos instrumentos.</t>
   </si>
   <si>
     <t xml:space="preserve">Ingreso</t>
@@ -2029,14 +2032,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
     <numFmt numFmtId="166" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="168" formatCode="mmm\-yy"/>
-    <numFmt numFmtId="169" formatCode="0.00"/>
-    <numFmt numFmtId="170" formatCode="General"/>
+    <numFmt numFmtId="169" formatCode="mm/dd/yy"/>
+    <numFmt numFmtId="170" formatCode="0.00"/>
+    <numFmt numFmtId="171" formatCode="General"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -2351,7 +2355,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="167">
+  <cellXfs count="162">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2888,6 +2892,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2908,31 +2920,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="10" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2952,22 +2952,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="10" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2980,11 +2964,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2996,7 +2980,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="10" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="10" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3004,7 +2988,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="11" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="11" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3174,9 +3158,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>163440</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>60840</xdr:rowOff>
+      <xdr:colOff>162720</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>400320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3189,8 +3173,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12909240" y="170280"/>
-          <a:ext cx="12341160" cy="5524200"/>
+          <a:off x="13092840" y="170280"/>
+          <a:ext cx="12359520" cy="5523480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3239,7 +3223,7 @@
     <tableColumn id="28" name="Visitas y observaciones ENE 2025"/>
     <tableColumn id="29" name="DL Tycon enero 2025"/>
     <tableColumn id="30" name="Observaciones octubre 2025"/>
-    <tableColumn id="31" name="DL Tycon octubre 20252"/>
+    <tableColumn id="31" name="DL Tycon octubre 2025"/>
   </tableColumns>
 </table>
 </file>
@@ -3250,7 +3234,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:AE111"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
@@ -3264,9 +3248,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="6.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="6.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="7.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="8.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="8.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="6.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="19" style="0" width="18.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="46.28"/>
@@ -3281,7 +3265,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="11.14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="45.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -12100,7 +12084,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AT101"/>
-  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.71"/>
@@ -24711,7 +24695,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AH20"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.85"/>
@@ -26550,7 +26534,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.85"/>
@@ -26746,8 +26730,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.47"/>
@@ -27077,26 +27061,62 @@
       <c r="G14" s="129"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="126" t="n">
+      <c r="A15" s="134" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="131" t="s">
+      <c r="B15" s="41" t="s">
         <v>559</v>
       </c>
-      <c r="C15" s="131" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="132" t="n">
+      <c r="C15" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="127" t="n">
         <v>45434</v>
       </c>
-      <c r="E15" s="131" t="s">
+      <c r="E15" s="41" t="s">
         <v>276</v>
       </c>
-      <c r="F15" s="133" t="s">
+      <c r="F15" s="128" t="s">
         <v>577</v>
       </c>
-      <c r="G15" s="129" t="s">
+      <c r="G15" s="134" t="s">
         <v>578</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="134" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="134" t="s">
+        <v>579</v>
+      </c>
+      <c r="C16" s="134" t="n">
+        <v>25</v>
+      </c>
+      <c r="D16" s="135" t="n">
+        <v>45615</v>
+      </c>
+      <c r="E16" s="134"/>
+      <c r="F16" s="134"/>
+      <c r="G16" s="134"/>
+    </row>
+    <row r="17" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="134" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="134" t="s">
+        <v>580</v>
+      </c>
+      <c r="C17" s="134" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="135" t="n">
+        <v>45932</v>
+      </c>
+      <c r="E17" s="134"/>
+      <c r="F17" s="134"/>
+      <c r="G17" s="134" t="s">
+        <v>581</v>
       </c>
     </row>
   </sheetData>
@@ -27131,87 +27151,88 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52.68"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="118" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="B1" s="119" t="s">
         <v>375</v>
       </c>
       <c r="C1" s="119" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="D1" s="120" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="121" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B2" s="123" t="n">
         <v>44658</v>
       </c>
       <c r="C2" s="122" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="41.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="121" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="B3" s="123" t="n">
         <v>44893</v>
       </c>
       <c r="C3" s="122" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="121" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="B4" s="123" t="n">
         <v>44951</v>
       </c>
       <c r="C4" s="122" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="41.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="121" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="B5" s="123" t="n">
         <v>44951</v>
       </c>
       <c r="C5" s="122" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="121" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="B6" s="123" t="n">
         <v>44951</v>
@@ -27220,54 +27241,54 @@
         <v>486</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="121" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B7" s="123" t="n">
         <v>45042</v>
       </c>
       <c r="C7" s="122" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="D7" s="125" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="121" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="B8" s="123" t="n">
         <v>45124</v>
       </c>
       <c r="C8" s="122" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="D8" s="125" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="121" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="B9" s="123" t="n">
         <v>45203</v>
       </c>
       <c r="C9" s="122" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="D9" s="125" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="41.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="121" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="B10" s="123" t="n">
         <v>45251</v>
@@ -27276,130 +27297,110 @@
         <v>486</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="134" t="s">
-        <v>604</v>
+      <c r="A11" s="136" t="s">
+        <v>607</v>
       </c>
       <c r="B11" s="123" t="n">
         <v>45320</v>
       </c>
       <c r="C11" s="122" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="D11" s="125" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="135" t="s">
-        <v>606</v>
-      </c>
-      <c r="B12" s="136" t="n">
+      <c r="A12" s="137" t="s">
+        <v>609</v>
+      </c>
+      <c r="B12" s="138" t="n">
         <v>45433</v>
       </c>
-      <c r="C12" s="137" t="s">
+      <c r="C12" s="139" t="s">
         <v>486</v>
       </c>
-      <c r="D12" s="138" t="s">
-        <v>607</v>
+      <c r="D12" s="140" t="s">
+        <v>610</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="54.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="139" t="s">
-        <v>608</v>
-      </c>
-      <c r="B13" s="140" t="n">
+      <c r="A13" s="137" t="s">
+        <v>611</v>
+      </c>
+      <c r="B13" s="138" t="n">
         <v>45615</v>
       </c>
-      <c r="C13" s="141" t="s">
+      <c r="C13" s="139" t="s">
         <v>486</v>
       </c>
-      <c r="D13" s="142" t="s">
-        <v>609</v>
+      <c r="D13" s="140" t="s">
+        <v>612</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="139" t="s">
-        <v>610</v>
-      </c>
-      <c r="B14" s="140" t="n">
+      <c r="A14" s="137" t="s">
+        <v>613</v>
+      </c>
+      <c r="B14" s="138" t="n">
         <v>45670</v>
       </c>
-      <c r="C14" s="141" t="s">
+      <c r="C14" s="139" t="s">
         <v>486</v>
       </c>
-      <c r="D14" s="142" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="139" t="s">
-        <v>610</v>
-      </c>
-      <c r="B15" s="143" t="n">
+      <c r="D14" s="140" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="137" t="s">
+        <v>615</v>
+      </c>
+      <c r="B15" s="123" t="n">
         <v>45932</v>
       </c>
-      <c r="C15" s="144" t="s">
+      <c r="C15" s="8" t="s">
         <v>486</v>
       </c>
-      <c r="D15" s="145" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="146" t="s">
-        <v>613</v>
-      </c>
-      <c r="B16" s="147" t="s">
+      <c r="D15" s="22" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="141" t="s">
+        <v>617</v>
+      </c>
+      <c r="B16" s="142" t="n">
+        <v>45817</v>
+      </c>
+      <c r="C16" s="143" t="s">
+        <v>486</v>
+      </c>
+      <c r="D16" s="144" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="137"/>
+      <c r="B17" s="123"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="22"/>
+    </row>
+    <row r="18" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="145" t="s">
+        <v>619</v>
+      </c>
+      <c r="B18" s="146" t="s">
         <v>246</v>
       </c>
-      <c r="C16" s="148" t="s">
-        <v>600</v>
-      </c>
-      <c r="D16" s="149"/>
-    </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="150" t="s">
-        <v>614</v>
-      </c>
-      <c r="B17" s="151" t="n">
-        <v>45817</v>
-      </c>
-      <c r="C17" s="152" t="s">
-        <v>600</v>
-      </c>
-      <c r="D17" s="153" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="150" t="s">
-        <v>616</v>
-      </c>
-      <c r="B18" s="147" t="n">
-        <v>45936</v>
-      </c>
-      <c r="C18" s="148" t="s">
-        <v>486</v>
-      </c>
-      <c r="D18" s="149"/>
-    </row>
-    <row r="19" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="150" t="s">
-        <v>617</v>
-      </c>
-      <c r="B19" s="151" t="n">
-        <v>46035</v>
-      </c>
-      <c r="C19" s="152" t="s">
-        <v>486</v>
-      </c>
-      <c r="D19" s="153" t="s">
-        <v>618</v>
-      </c>
+      <c r="C18" s="147" t="s">
+        <v>603</v>
+      </c>
+      <c r="D18" s="148"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -27419,7 +27420,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.57"/>
@@ -27428,32 +27429,32 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="154" t="n">
+      <c r="B2" s="149" t="n">
         <v>2023</v>
       </c>
-      <c r="C2" s="154"/>
-      <c r="D2" s="154" t="n">
+      <c r="C2" s="149"/>
+      <c r="D2" s="149" t="n">
         <v>2024</v>
       </c>
-      <c r="E2" s="154"/>
+      <c r="E2" s="149"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="10" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>621</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>620</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>619</v>
-      </c>
       <c r="E3" s="10" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B4" s="19" t="n">
         <v>50000</v>
@@ -27464,7 +27465,7 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B5" s="19" t="n">
         <v>396062.3496</v>
@@ -27475,7 +27476,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B6" s="19"/>
       <c r="C6" s="10" t="n">
@@ -27486,7 +27487,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="10" t="n">
@@ -27497,7 +27498,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="10" t="n">
@@ -27508,7 +27509,7 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B9" s="19"/>
       <c r="C9" s="10" t="n">
@@ -27519,7 +27520,7 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B10" s="19"/>
       <c r="C10" s="10" t="n">
@@ -27530,7 +27531,7 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B11" s="19"/>
       <c r="C11" s="10" t="n">
@@ -27540,8 +27541,8 @@
       <c r="E11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="155" t="s">
-        <v>629</v>
+      <c r="A12" s="150" t="s">
+        <v>630</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10" t="n">
@@ -27551,8 +27552,8 @@
       <c r="E12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="156" t="s">
-        <v>630</v>
+      <c r="A13" s="151" t="s">
+        <v>631</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10" t="n">
@@ -27562,8 +27563,8 @@
       <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="156" t="s">
-        <v>631</v>
+      <c r="A14" s="151" t="s">
+        <v>632</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="10" t="n">
@@ -27573,8 +27574,8 @@
       <c r="E14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="156" t="s">
-        <v>632</v>
+      <c r="A15" s="151" t="s">
+        <v>633</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10" t="n">
@@ -27584,8 +27585,8 @@
       <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="156" t="s">
-        <v>633</v>
+      <c r="A16" s="151" t="s">
+        <v>634</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10" t="n">
@@ -27595,8 +27596,8 @@
       <c r="E16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="156" t="s">
-        <v>634</v>
+      <c r="A17" s="151" t="s">
+        <v>635</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10" t="n">
@@ -27607,7 +27608,7 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10" t="n">
@@ -27618,12 +27619,12 @@
     </row>
     <row r="19" customFormat="false" ht="68.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="22" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
-      <c r="E19" s="157" t="n">
+      <c r="E19" s="152" t="n">
         <v>2094.5</v>
       </c>
       <c r="F19" s="0" t="n">
@@ -27633,12 +27634,12 @@
     </row>
     <row r="20" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
-      <c r="E20" s="158" t="n">
+      <c r="E20" s="153" t="n">
         <v>22220</v>
       </c>
       <c r="F20" s="0" t="n">
@@ -27648,12 +27649,12 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
-      <c r="E21" s="158" t="n">
+      <c r="E21" s="153" t="n">
         <v>600</v>
       </c>
       <c r="F21" s="0" t="n">
@@ -27663,12 +27664,12 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
-      <c r="E22" s="158" t="n">
+      <c r="E22" s="153" t="n">
         <v>21468.3</v>
       </c>
       <c r="F22" s="0" t="n">
@@ -27678,12 +27679,12 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
-      <c r="E23" s="158" t="n">
+      <c r="E23" s="153" t="n">
         <v>4640</v>
       </c>
       <c r="F23" s="0" t="n">
@@ -27693,7 +27694,7 @@
     </row>
     <row r="24" customFormat="false" ht="68.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="22" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -27707,8 +27708,8 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="68.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="138" t="s">
-        <v>642</v>
+      <c r="A25" s="140" t="s">
+        <v>643</v>
       </c>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
@@ -27723,7 +27724,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B26" s="19"/>
       <c r="C26" s="10"/>
@@ -27738,7 +27739,7 @@
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B27" s="19"/>
       <c r="C27" s="10"/>
@@ -27752,8 +27753,8 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="159" t="s">
-        <v>645</v>
+      <c r="A28" s="154" t="s">
+        <v>646</v>
       </c>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -27785,10 +27786,10 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="160" t="s">
-        <v>646</v>
-      </c>
-      <c r="B30" s="160"/>
+      <c r="A30" s="155" t="s">
+        <v>647</v>
+      </c>
+      <c r="B30" s="155"/>
       <c r="C30" s="39" t="n">
         <f aca="false">ABS(B29-C29)</f>
         <v>126807.5596</v>
@@ -27799,11 +27800,11 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="160" t="s">
-        <v>647</v>
-      </c>
-      <c r="B31" s="160"/>
-      <c r="C31" s="161" t="n">
+      <c r="A31" s="155" t="s">
+        <v>648</v>
+      </c>
+      <c r="B31" s="155"/>
+      <c r="C31" s="156" t="n">
         <f aca="false">SUM(E19:E28)</f>
         <v>75399.3</v>
       </c>
@@ -27813,11 +27814,11 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="162" t="s">
-        <v>648</v>
-      </c>
-      <c r="B32" s="162"/>
-      <c r="C32" s="163" t="n">
+      <c r="A32" s="157" t="s">
+        <v>649</v>
+      </c>
+      <c r="B32" s="157"/>
+      <c r="C32" s="158" t="n">
         <f aca="false">ABS(C30-C31)</f>
         <v>51408.2596</v>
       </c>
@@ -27828,12 +27829,12 @@
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="41.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="164" t="s">
-        <v>650</v>
+      <c r="A36" s="159" t="s">
+        <v>651</v>
       </c>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
@@ -27843,8 +27844,8 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="165" t="s">
-        <v>651</v>
+      <c r="A37" s="160" t="s">
+        <v>652</v>
       </c>
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
@@ -27854,8 +27855,8 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="165" t="s">
-        <v>652</v>
+      <c r="A38" s="160" t="s">
+        <v>653</v>
       </c>
       <c r="B38" s="54"/>
       <c r="C38" s="54"/>
@@ -27865,19 +27866,19 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="166" t="s">
-        <v>653</v>
-      </c>
-      <c r="C39" s="166"/>
-      <c r="D39" s="166"/>
+      <c r="B39" s="161" t="s">
+        <v>654</v>
+      </c>
+      <c r="C39" s="161"/>
+      <c r="D39" s="161"/>
       <c r="E39" s="10" t="n">
         <f aca="false">E36+E37+E38</f>
         <v>21280</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="160" t="s">
-        <v>654</v>
+      <c r="A42" s="155" t="s">
+        <v>655</v>
       </c>
       <c r="B42" s="20" t="n">
         <f aca="false">C32-E39</f>

</xml_diff>